<commit_message>
Split plastering and painting process groups
</commit_message>
<xml_diff>
--- a/process_merge_mapping.xlsx
+++ b/process_merge_mapping.xlsx
@@ -2896,12 +2896,12 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Wall plastering</t>
+          <t>Wall Painting</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>批盪/噴漿/油漆類</t>
+          <t>牆身油漆類</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -2929,10 +2929,14 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr"/>
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Wall plastering</t>
+        </is>
+      </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>批盪/噴漿/油漆類</t>
+          <t>牆身批盪/噴漿類</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -2960,10 +2964,14 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr"/>
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Wall plastering</t>
+        </is>
+      </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>批盪/噴漿/油漆類</t>
+          <t>牆身批盪/噴漿類</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -2991,10 +2999,14 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr"/>
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Wall plastering</t>
+        </is>
+      </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>批盪/噴漿/油漆類</t>
+          <t>牆身批盪/噴漿類</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -3053,10 +3065,14 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="inlineStr"/>
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Wall plastering</t>
+        </is>
+      </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>批盪/噴漿/油漆類</t>
+          <t>牆身批盪/噴漿類</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -3084,10 +3100,14 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr"/>
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Wall plastering</t>
+        </is>
+      </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>批盪/噴漿/油漆類</t>
+          <t>牆身批盪/噴漿類</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">

</xml_diff>